<commit_message>
feat(import): columna de validaciones por campo y precio 0 permitido
- Agrega una columna "Validaciones" al lado de "Descripción" en las tablas
  de plantilla de Servicios, Productos, Profesionales y Clientes, con las
  reglas que la importación aplica a cada campo (en.json + es.json).
- Quita la validación de precio mayor a cero para Servicios y Productos:
  precio 0 se importa; un precio negativo sigue rechazándose
  (IMPORT_ROW_PRICE_INVALID ahora dice "no puede ser negativo").
- Tests: unitarios de ServiceImportService, nuevo spec Playwright
  importar-columna-validaciones, y fixture/specs HU-51/HU-54 ajustados.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01SojQEhp2gXG4SR3UEoqEGM
</commit_message>
<xml_diff>
--- a/e2e/fixtures/import/servicios-import-mixto.xlsx
+++ b/e2e/fixtures/import/servicios-import-mixto.xlsx
@@ -504,12 +504,12 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Precio Cero</t>
+          <t>Precio Negativo</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>-100</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">

</xml_diff>